<commit_message>
Ajusta el documento de pruebas: agrega el repositorio y quita Mejoras v2
Cambios hechos en el Excel, ahora también en tools/generar_excel.py para
que no se pierdan al regenerarlo:
- Portada: nueva fila "Repositorio" con la URL de GitHub y columna B más
  ancha.
- Se elimina la hoja "Mejoras v2" y su fila en la tabla de contenido.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PTP_Carlos_Sanchez_13102026.xlsx
+++ b/PTP_Carlos_Sanchez_13102026.xlsx
@@ -13,7 +13,6 @@
     <sheet name="Esc2 - Modificar datos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Esc3 - Compra" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Hallazgos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Mejoras v2" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -740,7 +739,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="44.44140625" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -872,201 +871,201 @@
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Repositorio</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/C7julios/Automation_Qvision</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Resumen de la ejecución</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Escenario</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Hoja</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Duración (s)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="27" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>ESC-01</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Registro exitoso de usuario</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Esc1 - Registro</t>
         </is>
       </c>
-      <c r="D15" s="9">
+      <c r="D16" s="9">
         <f>'Esc1 - Registro'!B12</f>
         <v/>
       </c>
-      <c r="E15" s="10">
+      <c r="E16" s="10">
         <f>'Esc1 - Registro'!B13</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>ESC-02</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Modificación de datos del usuario registrado</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Esc2 - Modificar datos</t>
         </is>
       </c>
-      <c r="D16" s="9">
+      <c r="D17" s="9">
         <f>'Esc2 - Modificar datos'!B12</f>
         <v/>
       </c>
-      <c r="E16" s="10">
+      <c r="E17" s="10">
         <f>'Esc2 - Modificar datos'!B13</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>ESC-03</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Compra de producto (categoría Zapatos)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Esc3 - Compra</t>
         </is>
       </c>
-      <c r="D17" s="9">
+      <c r="D18" s="9">
         <f>'Esc3 - Compra'!B12</f>
         <v/>
       </c>
-      <c r="E17" s="10">
+      <c r="E18" s="10">
         <f>'Esc3 - Compra'!B13</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Escenarios ejecutados</t>
-        </is>
-      </c>
-      <c r="B18" s="12">
-        <f>COUNTA(A15:A17)</f>
-        <v/>
-      </c>
-    </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Escenarios exitosos</t>
+          <t>Escenarios ejecutados</t>
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(D15:D17,"Pasó")</f>
+        <f>COUNTA(A16:A18)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
+          <t>Escenarios exitosos</t>
+        </is>
+      </c>
+      <c r="B20" s="12">
+        <f>COUNTIF(D16:D18,"Pasó")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
           <t>% de éxito</t>
         </is>
       </c>
-      <c r="B20" s="13">
-        <f>IF(B18=0,0,B19/B18)</f>
+      <c r="B21" s="13">
+        <f>IF(B19=0,0,B20/B19)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Nota: los valores del resumen son fórmulas enlazadas a cada hoja de escenario; Excel los calcula al abrir.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Contenido del documento</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Hoja</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Contenido</t>
         </is>
       </c>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-    </row>
-    <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>Alcance y Estrategia</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>a) Objetivo, alcance, módulos, tipos y niveles de prueba, enfoque, herramientas, ambiente, datos, criterios, riesgos, roles, cronograma y entregables.</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="n"/>
     </row>
     <row r="27" ht="27" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Esc1 - Registro</t>
+          <t>Alcance y Estrategia</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>b) Solución del escenario 1: ficha, Gherkin, pasos automatizados con resultados, componentes Screenplay y evidencias.</t>
+          <t>a) Objetivo, alcance, módulos, tipos y niveles de prueba, enfoque, herramientas, ambiente, datos, criterios, riesgos, roles, cronograma y entregables.</t>
         </is>
       </c>
       <c r="C27" s="6" t="n"/>
@@ -1076,12 +1075,12 @@
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Esc2 - Modificar datos</t>
+          <t>Esc1 - Registro</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>b) Solución del escenario 2 (misma estructura).</t>
+          <t>b) Solución del escenario 1: ficha, Gherkin, pasos automatizados con resultados, componentes Screenplay y evidencias.</t>
         </is>
       </c>
       <c r="C28" s="6" t="n"/>
@@ -1091,12 +1090,12 @@
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Esc3 - Compra</t>
+          <t>Esc2 - Modificar datos</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>b) Solución del escenario 3 (misma estructura).</t>
+          <t>b) Solución del escenario 2 (misma estructura).</t>
         </is>
       </c>
       <c r="C29" s="6" t="n"/>
@@ -1106,12 +1105,12 @@
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Hallazgos</t>
+          <t>Esc3 - Compra</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Observaciones y posibles defectos detectados durante el diseño y la ejecución.</t>
+          <t>b) Solución del escenario 3 (misma estructura).</t>
         </is>
       </c>
       <c r="C30" s="6" t="n"/>
@@ -1121,12 +1120,12 @@
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Mejoras v2</t>
+          <t>Hallazgos</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Asesoría para la segunda versión del sitio orientada a los dolores de cada área.</t>
+          <t>Observaciones y posibles defectos detectados durante el diseño y la ejecución.</t>
         </is>
       </c>
       <c r="C31" s="6" t="n"/>
@@ -1136,22 +1135,22 @@
   </sheetData>
   <mergeCells count="19">
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A24:E24"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A25:E25"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B25:E25"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B12:E12"/>
     <mergeCell ref="B11:E11"/>
+    <mergeCell ref="A14:E14"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="B29:E29"/>
-    <mergeCell ref="A13:E13"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B28:E28"/>
   </mergeCells>
@@ -4607,175 +4606,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Asesoría para la versión 2 del sitio web</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cómo abordar las mejoras para beneficiar a las áreas de la empresa</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Área</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Dolor actual (v1 y aplicaciones aisladas)</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Mejora propuesta para la v2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40.5" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Mercadeo y Ventas</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Información de clientes y ventas en aplicaciones separadas; poca trazabilidad de campañas.</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>CRM integrado al sitio (clientes, newsletter, carritos abandonados), tablero de ventas por categoría/canal y cupones gestionados desde un solo lugar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40.5" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Costos</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Costos calculados manualmente y desconectados del precio publicado.</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Integrar el maestro de productos con costos (ERP) para calcular márgenes por referencia y alertar precios por debajo del costo (p. ej. en Outlet).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40.5" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Producción y logística</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Inventario y despachos en hojas o apps aisladas; productos agotados visibles.</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Sincronizar inventario en tiempo real (API WooCommerce ↔ ERP), integración con transportadoras, cálculo automático del envío por ciudad y seguimiento del pedido en Mi cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Facturación</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Facturas generadas manualmente a partir de los pedidos.</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Facturación electrónica DIAN automática al confirmar el pago, con los datos de facturación del checkout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40.5" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Contabilidad</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Registro manual de ventas, pagos y bonos de regalo.</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Conciliación automática de pagos de la pasarela y causación contable de ventas, devoluciones, créditos y bonos de regalo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="54" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Calidad (transversal)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Sin pruebas ni ambiente de pruebas.</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Pipeline CI/CD que ejecute esta suite en cada despliegue a staging, pruebas de API y de rendimiento antes de producción, y ampliar la automatización a todos los módulos de la matriz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Forma de abordarlo</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>1) Levantar en talleres con cada director los procesos y dolores (as-is). 2) Priorizar con matriz valor/esfuerzo. 3) Definir una arquitectura de integración (ERP como fuente única de productos, inventario, costos y facturación, con el sitio conectado por API). 4) Entregar en incrementos (MVP: inventario + facturación electrónica) con criterios de aceptación en Gherkin que alimenten directamente la automatización.</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="B12:C12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>